<commit_message>
Post PDR Actions - GUI updates, bug fixes
</commit_message>
<xml_diff>
--- a/data/defaultSRS.xlsx
+++ b/data/defaultSRS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId3"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="158">
   <si>
     <t xml:space="preserve">&lt;&lt;Project Name&gt;&gt;
 Software Requirements Specification </t>
@@ -275,13 +275,13 @@
 Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Justification</t>
+    <t xml:space="preserve">Requirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traceability to Parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale / Justification</t>
   </si>
   <si>
     <t xml:space="preserve">Priority</t>
@@ -413,20 +413,11 @@
 In order to integrate with the tagging and filtering in the requirements spreadsheet and TASTE, each requirement shall be linked to one of these specific areas.  This will be selected from a drop down list.</t>
   </si>
   <si>
-    <t xml:space="preserve">Requirement</t>
-  </si>
-  <si>
     <t xml:space="preserve">This is the field that holds the requirement text.  The requirement text will need to comply with the "key term" definitions given on sheet "3. Terms &amp; Definitions".
 The detail of what needs to go into the requirement is dependent upon the requirement type, and is specified as part of the ECSS standard.  Further details with respect to the ECSS expected response can be found in ECSS-E-ST-40C, Annex D, Section 5, 6th March 2009.</t>
   </si>
   <si>
-    <t xml:space="preserve">Traceability to Parent</t>
-  </si>
-  <si>
     <t xml:space="preserve">The ECSS standard states that traceability to the upper level specification is required.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rationale / Justification</t>
   </si>
   <si>
     <t xml:space="preserve">It is useful to record why a specific requirement has been created.  This allows assessment and analysis if needs or conflicts arise.</t>
@@ -1253,9 +1244,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>589320</xdr:colOff>
+      <xdr:colOff>588960</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1265,7 +1256,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10032120" y="1145520"/>
-          <a:ext cx="3831840" cy="2587320"/>
+          <a:ext cx="3831480" cy="2586960"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1295,9 +1286,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>430560</xdr:colOff>
+      <xdr:colOff>430200</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>4680</xdr:rowOff>
+      <xdr:rowOff>4320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1307,7 +1298,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4755600" y="99000"/>
-          <a:ext cx="4806720" cy="2437560"/>
+          <a:ext cx="4806360" cy="2437200"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1337,9 +1328,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>287280</xdr:colOff>
+      <xdr:colOff>286920</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>2476080</xdr:rowOff>
+      <xdr:rowOff>2475720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1349,7 +1340,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6387480" y="141120"/>
-          <a:ext cx="3591000" cy="2525400"/>
+          <a:ext cx="3590640" cy="2525040"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1379,9 +1370,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>179280</xdr:colOff>
+      <xdr:colOff>178920</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>133200</xdr:rowOff>
+      <xdr:rowOff>132840</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1391,7 +1382,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6462000" y="346320"/>
-          <a:ext cx="4115520" cy="1994760"/>
+          <a:ext cx="4115160" cy="1994400"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1421,9 +1412,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>570960</xdr:colOff>
+      <xdr:colOff>570600</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:rowOff>160560</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1433,7 +1424,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5775840" y="160920"/>
-          <a:ext cx="4125960" cy="7601040"/>
+          <a:ext cx="4125600" cy="7600680"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1463,9 +1454,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>209520</xdr:colOff>
+      <xdr:colOff>209160</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>46800</xdr:rowOff>
+      <xdr:rowOff>46440</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1475,7 +1466,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5913720" y="125280"/>
-          <a:ext cx="4168080" cy="1826640"/>
+          <a:ext cx="4167720" cy="1826280"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -1505,9 +1496,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>215280</xdr:colOff>
+      <xdr:colOff>214920</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>2171160</xdr:rowOff>
+      <xdr:rowOff>2170800</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1517,7 +1508,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6656760" y="135360"/>
-          <a:ext cx="5240520" cy="2226240"/>
+          <a:ext cx="5240160" cy="2225880"/>
         </a:xfrm>
         <a:noFill/>
         <a:ln w="0">
@@ -2405,35 +2396,35 @@
     </row>
     <row r="9" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="67" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="B9" s="68" t="s">
         <v>107</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="67" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="B10" s="68" t="s">
         <v>107</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="67" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="B11" s="68" t="s">
         <v>109</v>
       </c>
       <c r="C11" s="69" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2444,7 +2435,7 @@
         <v>109</v>
       </c>
       <c r="C12" s="69" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2455,18 +2446,18 @@
         <v>109</v>
       </c>
       <c r="C13" s="69" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="67" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B14" s="68" t="s">
         <v>109</v>
       </c>
       <c r="C14" s="69" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2477,40 +2468,40 @@
         <v>107</v>
       </c>
       <c r="C15" s="69" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="67" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B16" s="68" t="s">
         <v>109</v>
       </c>
       <c r="C16" s="69" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="67" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B17" s="68" t="s">
         <v>109</v>
       </c>
       <c r="C17" s="69" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="67" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B18" s="68" t="s">
         <v>109</v>
       </c>
       <c r="C18" s="69" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,30 +2512,30 @@
         <v>109</v>
       </c>
       <c r="C19" s="69" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="70" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B20" s="71" t="s">
         <v>109</v>
       </c>
       <c r="C20" s="72" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
     </row>
     <row r="23" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B23" s="23"/>
       <c r="C23" s="23"/>
@@ -2581,7 +2572,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
@@ -2607,7 +2598,7 @@
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="23" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B3" s="23"/>
       <c r="C3" s="23"/>
@@ -2733,7 +2724,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="73" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B24" s="73"/>
       <c r="C24" s="73"/>
@@ -2746,7 +2737,7 @@
     </row>
     <row r="25" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -2759,7 +2750,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B26" s="18" t="s">
         <v>32</v>
@@ -2767,7 +2758,7 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>34</v>
@@ -2775,7 +2766,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B28" s="18" t="s">
         <v>36</v>
@@ -2783,7 +2774,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B29" s="18" t="s">
         <v>38</v>
@@ -2791,62 +2782,62 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="73" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B42" s="73"/>
       <c r="C42" s="73"/>
@@ -2859,7 +2850,7 @@
     </row>
     <row r="43" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B43" s="23"/>
       <c r="C43" s="23"/>
@@ -2872,17 +2863,17 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2900,7 +2891,7 @@
     </row>
     <row r="49" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="23" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B49" s="23"/>
       <c r="C49" s="23"/>
@@ -2913,17 +2904,17 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="18" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="18" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>